<commit_message>
data: drop פרופ' בנעט; mark the remaining sourceless rows with a red asterisk
Those 23 lab tests were priced from the clinic catalog file with no price list behind them
and no way to verify them, so they are gone rather than published. Hill's Vet Essentials is
the only list left in that state; its marker is now a red * reading "ללא מקור", and both it
and the invoice-parsed ✻ are explained in the page footer instead of above the chips.

29 price lists, 5,697 items.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XoJGvA8cApVXFb92aBk3Fg
</commit_message>
<xml_diff>
--- a/downloads/labs.xlsx
+++ b/downloads/labs.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -529,24 +529,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>פרופ' בנעט</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>0</v>
-      </c>
-      <c r="C7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
+    <row r="8">
+      <c r="A8" t="inlineStr">
         <is>
           <t>נוסחה: עלות = מחיר ללא מע"מ × (1 − הנחה) × 1.18 ; מחיר ללקוח = עלות × (1 + מרווח %) + מרווח ₪</t>
         </is>
@@ -563,7 +547,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L813"/>
+  <dimension ref="A1:L790"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -40064,995 +40048,6 @@
         <v/>
       </c>
     </row>
-    <row r="791">
-      <c r="A791" t="inlineStr">
-        <is>
-          <t>פרופ' בנעט</t>
-        </is>
-      </c>
-      <c r="B791" t="inlineStr">
-        <is>
-          <t>Ehrlichia spp.</t>
-        </is>
-      </c>
-      <c r="C791" t="inlineStr">
-        <is>
-          <t>PCR</t>
-        </is>
-      </c>
-      <c r="F791" t="n">
-        <v>170.94</v>
-      </c>
-      <c r="G791" t="n">
-        <v>201.71</v>
-      </c>
-      <c r="H791">
-        <f>הגדרות!B7</f>
-        <v/>
-      </c>
-      <c r="I791">
-        <f>F791*(1-H791/100)*1.18</f>
-        <v/>
-      </c>
-      <c r="J791">
-        <f>הגדרות!C7</f>
-        <v/>
-      </c>
-      <c r="K791">
-        <f>הגדרות!D7</f>
-        <v/>
-      </c>
-      <c r="L791">
-        <f>I791*(1+J791/100)+K791</f>
-        <v/>
-      </c>
-    </row>
-    <row r="792">
-      <c r="A792" t="inlineStr">
-        <is>
-          <t>פרופ' בנעט</t>
-        </is>
-      </c>
-      <c r="B792" t="inlineStr">
-        <is>
-          <t>Babesia spp.</t>
-        </is>
-      </c>
-      <c r="C792" t="inlineStr">
-        <is>
-          <t>PCR</t>
-        </is>
-      </c>
-      <c r="F792" t="n">
-        <v>170.94</v>
-      </c>
-      <c r="G792" t="n">
-        <v>201.71</v>
-      </c>
-      <c r="H792">
-        <f>הגדרות!B7</f>
-        <v/>
-      </c>
-      <c r="I792">
-        <f>F792*(1-H792/100)*1.18</f>
-        <v/>
-      </c>
-      <c r="J792">
-        <f>הגדרות!C7</f>
-        <v/>
-      </c>
-      <c r="K792">
-        <f>הגדרות!D7</f>
-        <v/>
-      </c>
-      <c r="L792">
-        <f>I792*(1+J792/100)+K792</f>
-        <v/>
-      </c>
-    </row>
-    <row r="793">
-      <c r="A793" t="inlineStr">
-        <is>
-          <t>פרופ' בנעט</t>
-        </is>
-      </c>
-      <c r="B793" t="inlineStr">
-        <is>
-          <t>Hepatozoon spp.</t>
-        </is>
-      </c>
-      <c r="C793" t="inlineStr">
-        <is>
-          <t>PCR</t>
-        </is>
-      </c>
-      <c r="F793" t="n">
-        <v>170.94</v>
-      </c>
-      <c r="G793" t="n">
-        <v>201.71</v>
-      </c>
-      <c r="H793">
-        <f>הגדרות!B7</f>
-        <v/>
-      </c>
-      <c r="I793">
-        <f>F793*(1-H793/100)*1.18</f>
-        <v/>
-      </c>
-      <c r="J793">
-        <f>הגדרות!C7</f>
-        <v/>
-      </c>
-      <c r="K793">
-        <f>הגדרות!D7</f>
-        <v/>
-      </c>
-      <c r="L793">
-        <f>I793*(1+J793/100)+K793</f>
-        <v/>
-      </c>
-    </row>
-    <row r="794">
-      <c r="A794" t="inlineStr">
-        <is>
-          <t>פרופ' בנעט</t>
-        </is>
-      </c>
-      <c r="B794" t="inlineStr">
-        <is>
-          <t>Borrelia spp (Lyme)</t>
-        </is>
-      </c>
-      <c r="C794" t="inlineStr">
-        <is>
-          <t>PCR</t>
-        </is>
-      </c>
-      <c r="F794" t="n">
-        <v>170.94</v>
-      </c>
-      <c r="G794" t="n">
-        <v>201.71</v>
-      </c>
-      <c r="H794">
-        <f>הגדרות!B7</f>
-        <v/>
-      </c>
-      <c r="I794">
-        <f>F794*(1-H794/100)*1.18</f>
-        <v/>
-      </c>
-      <c r="J794">
-        <f>הגדרות!C7</f>
-        <v/>
-      </c>
-      <c r="K794">
-        <f>הגדרות!D7</f>
-        <v/>
-      </c>
-      <c r="L794">
-        <f>I794*(1+J794/100)+K794</f>
-        <v/>
-      </c>
-    </row>
-    <row r="795">
-      <c r="A795" t="inlineStr">
-        <is>
-          <t>פרופ' בנעט</t>
-        </is>
-      </c>
-      <c r="B795" t="inlineStr">
-        <is>
-          <t>Rickettsia spp.</t>
-        </is>
-      </c>
-      <c r="C795" t="inlineStr">
-        <is>
-          <t>PCR</t>
-        </is>
-      </c>
-      <c r="F795" t="n">
-        <v>170.94</v>
-      </c>
-      <c r="G795" t="n">
-        <v>201.71</v>
-      </c>
-      <c r="H795">
-        <f>הגדרות!B7</f>
-        <v/>
-      </c>
-      <c r="I795">
-        <f>F795*(1-H795/100)*1.18</f>
-        <v/>
-      </c>
-      <c r="J795">
-        <f>הגדרות!C7</f>
-        <v/>
-      </c>
-      <c r="K795">
-        <f>הגדרות!D7</f>
-        <v/>
-      </c>
-      <c r="L795">
-        <f>I795*(1+J795/100)+K795</f>
-        <v/>
-      </c>
-    </row>
-    <row r="796">
-      <c r="A796" t="inlineStr">
-        <is>
-          <t>פרופ' בנעט</t>
-        </is>
-      </c>
-      <c r="B796" t="inlineStr">
-        <is>
-          <t>Bartonella spp.</t>
-        </is>
-      </c>
-      <c r="C796" t="inlineStr">
-        <is>
-          <t>PCR</t>
-        </is>
-      </c>
-      <c r="F796" t="n">
-        <v>170.94</v>
-      </c>
-      <c r="G796" t="n">
-        <v>201.71</v>
-      </c>
-      <c r="H796">
-        <f>הגדרות!B7</f>
-        <v/>
-      </c>
-      <c r="I796">
-        <f>F796*(1-H796/100)*1.18</f>
-        <v/>
-      </c>
-      <c r="J796">
-        <f>הגדרות!C7</f>
-        <v/>
-      </c>
-      <c r="K796">
-        <f>הגדרות!D7</f>
-        <v/>
-      </c>
-      <c r="L796">
-        <f>I796*(1+J796/100)+K796</f>
-        <v/>
-      </c>
-    </row>
-    <row r="797">
-      <c r="A797" t="inlineStr">
-        <is>
-          <t>פרופ' בנעט</t>
-        </is>
-      </c>
-      <c r="B797" t="inlineStr">
-        <is>
-          <t>Mycoplasma Hemofelis/Hemocanis</t>
-        </is>
-      </c>
-      <c r="C797" t="inlineStr">
-        <is>
-          <t>PCR</t>
-        </is>
-      </c>
-      <c r="F797" t="n">
-        <v>170.94</v>
-      </c>
-      <c r="G797" t="n">
-        <v>201.71</v>
-      </c>
-      <c r="H797">
-        <f>הגדרות!B7</f>
-        <v/>
-      </c>
-      <c r="I797">
-        <f>F797*(1-H797/100)*1.18</f>
-        <v/>
-      </c>
-      <c r="J797">
-        <f>הגדרות!C7</f>
-        <v/>
-      </c>
-      <c r="K797">
-        <f>הגדרות!D7</f>
-        <v/>
-      </c>
-      <c r="L797">
-        <f>I797*(1+J797/100)+K797</f>
-        <v/>
-      </c>
-    </row>
-    <row r="798">
-      <c r="A798" t="inlineStr">
-        <is>
-          <t>פרופ' בנעט</t>
-        </is>
-      </c>
-      <c r="B798" t="inlineStr">
-        <is>
-          <t>Canine Parvo Virus</t>
-        </is>
-      </c>
-      <c r="C798" t="inlineStr">
-        <is>
-          <t>PCR</t>
-        </is>
-      </c>
-      <c r="F798" t="n">
-        <v>170.94</v>
-      </c>
-      <c r="G798" t="n">
-        <v>201.71</v>
-      </c>
-      <c r="H798">
-        <f>הגדרות!B7</f>
-        <v/>
-      </c>
-      <c r="I798">
-        <f>F798*(1-H798/100)*1.18</f>
-        <v/>
-      </c>
-      <c r="J798">
-        <f>הגדרות!C7</f>
-        <v/>
-      </c>
-      <c r="K798">
-        <f>הגדרות!D7</f>
-        <v/>
-      </c>
-      <c r="L798">
-        <f>I798*(1+J798/100)+K798</f>
-        <v/>
-      </c>
-    </row>
-    <row r="799">
-      <c r="A799" t="inlineStr">
-        <is>
-          <t>פרופ' בנעט</t>
-        </is>
-      </c>
-      <c r="B799" t="inlineStr">
-        <is>
-          <t>Canine Distemper Virus</t>
-        </is>
-      </c>
-      <c r="C799" t="inlineStr">
-        <is>
-          <t>PCR</t>
-        </is>
-      </c>
-      <c r="F799" t="n">
-        <v>222.22</v>
-      </c>
-      <c r="G799" t="n">
-        <v>262.22</v>
-      </c>
-      <c r="H799">
-        <f>הגדרות!B7</f>
-        <v/>
-      </c>
-      <c r="I799">
-        <f>F799*(1-H799/100)*1.18</f>
-        <v/>
-      </c>
-      <c r="J799">
-        <f>הגדרות!C7</f>
-        <v/>
-      </c>
-      <c r="K799">
-        <f>הגדרות!D7</f>
-        <v/>
-      </c>
-      <c r="L799">
-        <f>I799*(1+J799/100)+K799</f>
-        <v/>
-      </c>
-    </row>
-    <row r="800">
-      <c r="A800" t="inlineStr">
-        <is>
-          <t>פרופ' בנעט</t>
-        </is>
-      </c>
-      <c r="B800" t="inlineStr">
-        <is>
-          <t>Canine Herpes Virus</t>
-        </is>
-      </c>
-      <c r="C800" t="inlineStr">
-        <is>
-          <t>PCR</t>
-        </is>
-      </c>
-      <c r="F800" t="n">
-        <v>170.94</v>
-      </c>
-      <c r="G800" t="n">
-        <v>201.71</v>
-      </c>
-      <c r="H800">
-        <f>הגדרות!B7</f>
-        <v/>
-      </c>
-      <c r="I800">
-        <f>F800*(1-H800/100)*1.18</f>
-        <v/>
-      </c>
-      <c r="J800">
-        <f>הגדרות!C7</f>
-        <v/>
-      </c>
-      <c r="K800">
-        <f>הגדרות!D7</f>
-        <v/>
-      </c>
-      <c r="L800">
-        <f>I800*(1+J800/100)+K800</f>
-        <v/>
-      </c>
-    </row>
-    <row r="801">
-      <c r="A801" t="inlineStr">
-        <is>
-          <t>פרופ' בנעט</t>
-        </is>
-      </c>
-      <c r="B801" t="inlineStr">
-        <is>
-          <t>Leishmania</t>
-        </is>
-      </c>
-      <c r="C801" t="inlineStr">
-        <is>
-          <t>PCR</t>
-        </is>
-      </c>
-      <c r="F801" t="n">
-        <v>170.94</v>
-      </c>
-      <c r="G801" t="n">
-        <v>201.71</v>
-      </c>
-      <c r="H801">
-        <f>הגדרות!B7</f>
-        <v/>
-      </c>
-      <c r="I801">
-        <f>F801*(1-H801/100)*1.18</f>
-        <v/>
-      </c>
-      <c r="J801">
-        <f>הגדרות!C7</f>
-        <v/>
-      </c>
-      <c r="K801">
-        <f>הגדרות!D7</f>
-        <v/>
-      </c>
-      <c r="L801">
-        <f>I801*(1+J801/100)+K801</f>
-        <v/>
-      </c>
-    </row>
-    <row r="802">
-      <c r="A802" t="inlineStr">
-        <is>
-          <t>פרופ' בנעט</t>
-        </is>
-      </c>
-      <c r="B802" t="inlineStr">
-        <is>
-          <t>Corona Virus</t>
-        </is>
-      </c>
-      <c r="C802" t="inlineStr">
-        <is>
-          <t>PCR</t>
-        </is>
-      </c>
-      <c r="F802" t="n">
-        <v>222.22</v>
-      </c>
-      <c r="G802" t="n">
-        <v>262.22</v>
-      </c>
-      <c r="H802">
-        <f>הגדרות!B7</f>
-        <v/>
-      </c>
-      <c r="I802">
-        <f>F802*(1-H802/100)*1.18</f>
-        <v/>
-      </c>
-      <c r="J802">
-        <f>הגדרות!C7</f>
-        <v/>
-      </c>
-      <c r="K802">
-        <f>הגדרות!D7</f>
-        <v/>
-      </c>
-      <c r="L802">
-        <f>I802*(1+J802/100)+K802</f>
-        <v/>
-      </c>
-    </row>
-    <row r="803">
-      <c r="A803" t="inlineStr">
-        <is>
-          <t>פרופ' בנעט</t>
-        </is>
-      </c>
-      <c r="B803" t="inlineStr">
-        <is>
-          <t>Corona Virus (FIP)</t>
-        </is>
-      </c>
-      <c r="C803" t="inlineStr">
-        <is>
-          <t>PCR</t>
-        </is>
-      </c>
-      <c r="F803" t="n">
-        <v>222.22</v>
-      </c>
-      <c r="G803" t="n">
-        <v>262.22</v>
-      </c>
-      <c r="H803">
-        <f>הגדרות!B7</f>
-        <v/>
-      </c>
-      <c r="I803">
-        <f>F803*(1-H803/100)*1.18</f>
-        <v/>
-      </c>
-      <c r="J803">
-        <f>הגדרות!C7</f>
-        <v/>
-      </c>
-      <c r="K803">
-        <f>הגדרות!D7</f>
-        <v/>
-      </c>
-      <c r="L803">
-        <f>I803*(1+J803/100)+K803</f>
-        <v/>
-      </c>
-    </row>
-    <row r="804">
-      <c r="A804" t="inlineStr">
-        <is>
-          <t>פרופ' בנעט</t>
-        </is>
-      </c>
-      <c r="B804" t="inlineStr">
-        <is>
-          <t>Salmonella sp.</t>
-        </is>
-      </c>
-      <c r="C804" t="inlineStr">
-        <is>
-          <t>PCR</t>
-        </is>
-      </c>
-      <c r="F804" t="n">
-        <v>170.94</v>
-      </c>
-      <c r="G804" t="n">
-        <v>201.71</v>
-      </c>
-      <c r="H804">
-        <f>הגדרות!B7</f>
-        <v/>
-      </c>
-      <c r="I804">
-        <f>F804*(1-H804/100)*1.18</f>
-        <v/>
-      </c>
-      <c r="J804">
-        <f>הגדרות!C7</f>
-        <v/>
-      </c>
-      <c r="K804">
-        <f>הגדרות!D7</f>
-        <v/>
-      </c>
-      <c r="L804">
-        <f>I804*(1+J804/100)+K804</f>
-        <v/>
-      </c>
-    </row>
-    <row r="805">
-      <c r="A805" t="inlineStr">
-        <is>
-          <t>פרופ' בנעט</t>
-        </is>
-      </c>
-      <c r="B805" t="inlineStr">
-        <is>
-          <t>Dirofilaria Immitis / Repens</t>
-        </is>
-      </c>
-      <c r="C805" t="inlineStr">
-        <is>
-          <t>PCR</t>
-        </is>
-      </c>
-      <c r="F805" t="n">
-        <v>170.94</v>
-      </c>
-      <c r="G805" t="n">
-        <v>201.71</v>
-      </c>
-      <c r="H805">
-        <f>הגדרות!B7</f>
-        <v/>
-      </c>
-      <c r="I805">
-        <f>F805*(1-H805/100)*1.18</f>
-        <v/>
-      </c>
-      <c r="J805">
-        <f>הגדרות!C7</f>
-        <v/>
-      </c>
-      <c r="K805">
-        <f>הגדרות!D7</f>
-        <v/>
-      </c>
-      <c r="L805">
-        <f>I805*(1+J805/100)+K805</f>
-        <v/>
-      </c>
-    </row>
-    <row r="806">
-      <c r="A806" t="inlineStr">
-        <is>
-          <t>פרופ' בנעט</t>
-        </is>
-      </c>
-      <c r="B806" t="inlineStr">
-        <is>
-          <t>Neospora Caninum</t>
-        </is>
-      </c>
-      <c r="C806" t="inlineStr">
-        <is>
-          <t>PCR</t>
-        </is>
-      </c>
-      <c r="F806" t="n">
-        <v>170.94</v>
-      </c>
-      <c r="G806" t="n">
-        <v>201.71</v>
-      </c>
-      <c r="H806">
-        <f>הגדרות!B7</f>
-        <v/>
-      </c>
-      <c r="I806">
-        <f>F806*(1-H806/100)*1.18</f>
-        <v/>
-      </c>
-      <c r="J806">
-        <f>הגדרות!C7</f>
-        <v/>
-      </c>
-      <c r="K806">
-        <f>הגדרות!D7</f>
-        <v/>
-      </c>
-      <c r="L806">
-        <f>I806*(1+J806/100)+K806</f>
-        <v/>
-      </c>
-    </row>
-    <row r="807">
-      <c r="A807" t="inlineStr">
-        <is>
-          <t>פרופ' בנעט</t>
-        </is>
-      </c>
-      <c r="B807" t="inlineStr">
-        <is>
-          <t>Feline Herpes Virus</t>
-        </is>
-      </c>
-      <c r="C807" t="inlineStr">
-        <is>
-          <t>PCR</t>
-        </is>
-      </c>
-      <c r="F807" t="n">
-        <v>170.94</v>
-      </c>
-      <c r="G807" t="n">
-        <v>201.71</v>
-      </c>
-      <c r="H807">
-        <f>הגדרות!B7</f>
-        <v/>
-      </c>
-      <c r="I807">
-        <f>F807*(1-H807/100)*1.18</f>
-        <v/>
-      </c>
-      <c r="J807">
-        <f>הגדרות!C7</f>
-        <v/>
-      </c>
-      <c r="K807">
-        <f>הגדרות!D7</f>
-        <v/>
-      </c>
-      <c r="L807">
-        <f>I807*(1+J807/100)+K807</f>
-        <v/>
-      </c>
-    </row>
-    <row r="808">
-      <c r="A808" t="inlineStr">
-        <is>
-          <t>פרופ' בנעט</t>
-        </is>
-      </c>
-      <c r="B808" t="inlineStr">
-        <is>
-          <t>Feline Leukemia Virus (FeLV)</t>
-        </is>
-      </c>
-      <c r="C808" t="inlineStr">
-        <is>
-          <t>PCR</t>
-        </is>
-      </c>
-      <c r="F808" t="n">
-        <v>170.94</v>
-      </c>
-      <c r="G808" t="n">
-        <v>201.71</v>
-      </c>
-      <c r="H808">
-        <f>הגדרות!B7</f>
-        <v/>
-      </c>
-      <c r="I808">
-        <f>F808*(1-H808/100)*1.18</f>
-        <v/>
-      </c>
-      <c r="J808">
-        <f>הגדרות!C7</f>
-        <v/>
-      </c>
-      <c r="K808">
-        <f>הגדרות!D7</f>
-        <v/>
-      </c>
-      <c r="L808">
-        <f>I808*(1+J808/100)+K808</f>
-        <v/>
-      </c>
-    </row>
-    <row r="809">
-      <c r="A809" t="inlineStr">
-        <is>
-          <t>פרופ' בנעט</t>
-        </is>
-      </c>
-      <c r="B809" t="inlineStr">
-        <is>
-          <t>Feline Immunodeficiency Virus (FIV)</t>
-        </is>
-      </c>
-      <c r="C809" t="inlineStr">
-        <is>
-          <t>PCR</t>
-        </is>
-      </c>
-      <c r="F809" t="n">
-        <v>170.94</v>
-      </c>
-      <c r="G809" t="n">
-        <v>201.71</v>
-      </c>
-      <c r="H809">
-        <f>הגדרות!B7</f>
-        <v/>
-      </c>
-      <c r="I809">
-        <f>F809*(1-H809/100)*1.18</f>
-        <v/>
-      </c>
-      <c r="J809">
-        <f>הגדרות!C7</f>
-        <v/>
-      </c>
-      <c r="K809">
-        <f>הגדרות!D7</f>
-        <v/>
-      </c>
-      <c r="L809">
-        <f>I809*(1+J809/100)+K809</f>
-        <v/>
-      </c>
-    </row>
-    <row r="810">
-      <c r="A810" t="inlineStr">
-        <is>
-          <t>פרופ' בנעט</t>
-        </is>
-      </c>
-      <c r="B810" t="inlineStr">
-        <is>
-          <t>Toxoplasma</t>
-        </is>
-      </c>
-      <c r="C810" t="inlineStr">
-        <is>
-          <t>PCR</t>
-        </is>
-      </c>
-      <c r="F810" t="n">
-        <v>170.94</v>
-      </c>
-      <c r="G810" t="n">
-        <v>201.71</v>
-      </c>
-      <c r="H810">
-        <f>הגדרות!B7</f>
-        <v/>
-      </c>
-      <c r="I810">
-        <f>F810*(1-H810/100)*1.18</f>
-        <v/>
-      </c>
-      <c r="J810">
-        <f>הגדרות!C7</f>
-        <v/>
-      </c>
-      <c r="K810">
-        <f>הגדרות!D7</f>
-        <v/>
-      </c>
-      <c r="L810">
-        <f>I810*(1+J810/100)+K810</f>
-        <v/>
-      </c>
-    </row>
-    <row r="811">
-      <c r="A811" t="inlineStr">
-        <is>
-          <t>פרופ' בנעט</t>
-        </is>
-      </c>
-      <c r="B811" t="inlineStr">
-        <is>
-          <t>Panleukopenia Parvo Virus</t>
-        </is>
-      </c>
-      <c r="C811" t="inlineStr">
-        <is>
-          <t>PCR</t>
-        </is>
-      </c>
-      <c r="F811" t="n">
-        <v>170.94</v>
-      </c>
-      <c r="G811" t="n">
-        <v>201.71</v>
-      </c>
-      <c r="H811">
-        <f>הגדרות!B7</f>
-        <v/>
-      </c>
-      <c r="I811">
-        <f>F811*(1-H811/100)*1.18</f>
-        <v/>
-      </c>
-      <c r="J811">
-        <f>הגדרות!C7</f>
-        <v/>
-      </c>
-      <c r="K811">
-        <f>הגדרות!D7</f>
-        <v/>
-      </c>
-      <c r="L811">
-        <f>I811*(1+J811/100)+K811</f>
-        <v/>
-      </c>
-    </row>
-    <row r="812">
-      <c r="A812" t="inlineStr">
-        <is>
-          <t>פרופ' בנעט</t>
-        </is>
-      </c>
-      <c r="B812" t="inlineStr">
-        <is>
-          <t>Feline Calici Virus</t>
-        </is>
-      </c>
-      <c r="C812" t="inlineStr">
-        <is>
-          <t>PCR</t>
-        </is>
-      </c>
-      <c r="F812" t="n">
-        <v>222.22</v>
-      </c>
-      <c r="G812" t="n">
-        <v>262.22</v>
-      </c>
-      <c r="H812">
-        <f>הגדרות!B7</f>
-        <v/>
-      </c>
-      <c r="I812">
-        <f>F812*(1-H812/100)*1.18</f>
-        <v/>
-      </c>
-      <c r="J812">
-        <f>הגדרות!C7</f>
-        <v/>
-      </c>
-      <c r="K812">
-        <f>הגדרות!D7</f>
-        <v/>
-      </c>
-      <c r="L812">
-        <f>I812*(1+J812/100)+K812</f>
-        <v/>
-      </c>
-    </row>
-    <row r="813">
-      <c r="A813" t="inlineStr">
-        <is>
-          <t>פרופ' בנעט</t>
-        </is>
-      </c>
-      <c r="B813" t="inlineStr">
-        <is>
-          <t>Chlamydophila Felis</t>
-        </is>
-      </c>
-      <c r="C813" t="inlineStr">
-        <is>
-          <t>PCR</t>
-        </is>
-      </c>
-      <c r="F813" t="n">
-        <v>170.94</v>
-      </c>
-      <c r="G813" t="n">
-        <v>201.71</v>
-      </c>
-      <c r="H813">
-        <f>הגדרות!B7</f>
-        <v/>
-      </c>
-      <c r="I813">
-        <f>F813*(1-H813/100)*1.18</f>
-        <v/>
-      </c>
-      <c r="J813">
-        <f>הגדרות!C7</f>
-        <v/>
-      </c>
-      <c r="K813">
-        <f>הגדרות!D7</f>
-        <v/>
-      </c>
-      <c r="L813">
-        <f>I813*(1+J813/100)+K813</f>
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>